<commit_message>
Leads: 2026-10-22 13:45 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,182 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HVAC Contractor | Colorado Springs, CO | 719-290-2746</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>affordableaircarehvac.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.affordableaircarehvac.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Affordable Air</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>prchecketts@aol.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>719-290-2746</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HVAC contractor Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A &amp; Z Mechanical</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>aandzmechanical.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://aandzmechanical.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Colorado Springs</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>office@aandzmechanicalinc.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>719-204-6867</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>HVAC contractor Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ComfortMAX Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>comfortmaxheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://comfortmaxheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@comfortmaxheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(719) 284-4386</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>HVAC contractor Colorado Springs CO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-22 13:48 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,6 @@
           <t>https://comfortmaxheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>info@comfortmaxheatingandcooling.com</t>
@@ -794,6 +793,62 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rebates</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cwlp.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.cwlp.com/ServicesHome/ServicesInformation/AllRebates.aspx</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>nrgxprts@cwlp.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>217.789.2070</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Springfield IL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>heat pump installation Springfield IL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-22 19:53 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,6 @@
           <t>https://www.cwlp.com/ServicesHome/ServicesInformation/AllRebates.aspx</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>nrgxprts@cwlp.com</t>
@@ -849,6 +848,62 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Energy Resource Group</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>metalroofspringfield.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.metalroofspringfield.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofspringfield.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>217-203-8969</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Springfield IL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>96</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Springfield IL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-22 20:01 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -874,7 +874,6 @@
           <t>https://www.metalroofspringfield.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>moreinfo@metalroofspringfield.com</t>
@@ -904,6 +903,122 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rail Roofing Group</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>railroofingpa.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://railroofingpa.com/service-areas/reading</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>rail3construction@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(570) 996-7357</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Reading PA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofer Reading PA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Professional Roofing Services in Reading, PA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>leddyroofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://leddyroofing.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Berks County</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>rayleddy16@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(484) 955-1312</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Reading PA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofer Reading PA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-22 20:09 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -929,7 +929,6 @@
           <t>https://railroofingpa.com/service-areas/reading</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>rail3construction@gmail.com</t>
@@ -1019,6 +1018,66 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Cary, NC | Licensed &amp; Available 24/7</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>plumbingexpertscary.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://plumbingexpertscary.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Blog Plumbing</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>contact@plumbingexpertscary.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(984) 237-6514</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Cary NC</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>emergency plumber Cary NC</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-22 20:12 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1083,6 +1083,122 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>gilbertaz plumbers</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>gilbertazplumbers.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://gilbertazplumbers.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Service Call</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>info@gilbertazplumbers.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>844-973-0400</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumbing company Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A&amp;K Plumbing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>akplumbingandmechanical.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.akplumbingandmechanical.com/gilbert-az</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>office@akplumbingandmechanical.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>602-905-3990</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>plumbing company Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-22 20:16 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-22.xlsx
+++ b/output/leads_2026-10-22.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1164,7 +1164,6 @@
           <t>https://www.akplumbingandmechanical.com/gilbert-az</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>office@akplumbingandmechanical.com</t>
@@ -1194,6 +1193,186 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Community Roofing Texas</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>communityroofingtexas.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://communityroofingtexas.com/roofing-contractor-pearland</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Free Estimate</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@communityrfg.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>713-364-4525</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Pearland TX</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof replacement Pearland TX</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lord Plumbing Company</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>lordplumbingcompany.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://lordplumbingcompany.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Lord Plumbing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>mihaisinaia1@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(757) 390-6235</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumbing company Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tell Projects TX</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>pearland.tellprojectstx.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://pearland.tellprojectstx.com/services/roofing-services.html</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Get Free</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@tellprojectstx.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(832) 301-9182</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Pearland TX</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roof replacement Pearland TX</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-22</t>
         </is>

</xml_diff>